<commit_message>
fix code mode value show error
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-d8ae17.o</t>
+    <t>lto-llvm-3e4af7.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -243,7 +243,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-d8ae17.o</c:v>
+                  <c:v>lto-llvm-3e4af7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -338,7 +338,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-d8ae17.o</c:v>
+                  <c:v>lto-llvm-3e4af7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -452,106 +452,106 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>93.97653961181641</c:v>
+                  <c:v>94.00738525390625</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.394596576690674</c:v>
+                  <c:v>2.382333278656006</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5744756460189819</c:v>
+                  <c:v>0.5715336799621582</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4749377965927124</c:v>
+                  <c:v>0.4725055396556854</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3298968970775604</c:v>
+                  <c:v>0.3282074630260468</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3242090344429016</c:v>
+                  <c:v>0.3225486874580383</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2644863128662109</c:v>
+                  <c:v>0.2631318271160126</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2502666115760803</c:v>
+                  <c:v>0.2489849627017975</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1564166396856308</c:v>
+                  <c:v>0.1556155979633331</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1421969383955002</c:v>
+                  <c:v>0.141468733549118</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08816210180521011</c:v>
+                  <c:v>0.08771061152219772</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.0796302855014801</c:v>
+                  <c:v>0.07922248542308807</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.0767863467335701</c:v>
+                  <c:v>0.07639311254024506</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07109846919775009</c:v>
+                  <c:v>0.07073436677455902</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.07109846919775009</c:v>
+                  <c:v>0.07073436677455902</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.06825453042984009</c:v>
+                  <c:v>0.06790498644113541</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.05687877535820007</c:v>
+                  <c:v>0.05658749118447304</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.05403483659029007</c:v>
+                  <c:v>0.05375811830163002</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.05119089782238007</c:v>
+                  <c:v>0.0509287416934967</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.05119089782238007</c:v>
+                  <c:v>0.0509287416934967</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04834695905447006</c:v>
+                  <c:v>0.04809936881065369</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.04550302028656006</c:v>
+                  <c:v>0.04526999220252037</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.04265908151865006</c:v>
+                  <c:v>0.04244061931967735</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.04265908151865006</c:v>
+                  <c:v>0.04244061931967735</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.03981514275074005</c:v>
+                  <c:v>0.03961124271154404</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03981514275074005</c:v>
+                  <c:v>0.03961124271154404</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03981514275074005</c:v>
+                  <c:v>0.03961124271154404</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03981514275074005</c:v>
+                  <c:v>0.03961124271154404</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.03697120398283005</c:v>
+                  <c:v>0.03678186982870102</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02559544891119003</c:v>
+                  <c:v>0.02546437084674835</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01421969383955002</c:v>
+                  <c:v>0.01414687279611826</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01137575507164002</c:v>
+                  <c:v>0.01131749805063009</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01137575507164002</c:v>
+                  <c:v>0.01131749805063009</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.005687877535820007</c:v>
+                  <c:v>0.005658749025315046</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -1024,10 +1024,10 @@
         <v>11411</v>
       </c>
       <c r="D3" s="1">
-        <v>66089</v>
+        <v>66451</v>
       </c>
       <c r="E3" s="1">
-        <v>65844</v>
+        <v>66206</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1151,16 +1151,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>93.97653961181641</v>
+        <v>94.00738525390625</v>
       </c>
       <c r="C3" s="1">
-        <v>66089</v>
+        <v>66451</v>
       </c>
       <c r="D3" s="1">
         <v>11411</v>
       </c>
       <c r="E3" s="1">
-        <v>65844</v>
+        <v>66206</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1177,7 +1177,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.394596576690674</v>
+        <v>2.382333278656006</v>
       </c>
       <c r="C4" s="1">
         <v>1684</v>
@@ -1203,7 +1203,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5744756460189819</v>
+        <v>0.5715336799621582</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.4749377965927124</v>
+        <v>0.4725055396556854</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1255,7 +1255,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.3298968970775604</v>
+        <v>0.3282074630260468</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1281,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3242090344429016</v>
+        <v>0.3225486874580383</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1307,7 +1307,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.2644863128662109</v>
+        <v>0.2631318271160126</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1333,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2502666115760803</v>
+        <v>0.2489849627017975</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1359,7 +1359,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1564166396856308</v>
+        <v>0.1556155979633331</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1385,7 +1385,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.1421969383955002</v>
+        <v>0.141468733549118</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1411,7 +1411,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08816210180521011</v>
+        <v>0.08771061152219772</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1437,7 +1437,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.0796302855014801</v>
+        <v>0.07922248542308807</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1463,7 +1463,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.0767863467335701</v>
+        <v>0.07639311254024506</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1489,7 +1489,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07109846919775009</v>
+        <v>0.07073436677455902</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1515,7 +1515,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.07109846919775009</v>
+        <v>0.07073436677455902</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1541,7 +1541,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.06825453042984009</v>
+        <v>0.06790498644113541</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1567,7 +1567,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.05687877535820007</v>
+        <v>0.05658749118447304</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.05403483659029007</v>
+        <v>0.05375811830163002</v>
       </c>
       <c r="C20" s="1">
         <v>38</v>
@@ -1619,7 +1619,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.05119089782238007</v>
+        <v>0.0509287416934967</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1645,7 +1645,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.05119089782238007</v>
+        <v>0.0509287416934967</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1671,7 +1671,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04834695905447006</v>
+        <v>0.04809936881065369</v>
       </c>
       <c r="C23" s="1">
         <v>34</v>
@@ -1697,7 +1697,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.04550302028656006</v>
+        <v>0.04526999220252037</v>
       </c>
       <c r="C24" s="1">
         <v>32</v>
@@ -1723,7 +1723,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.04265908151865006</v>
+        <v>0.04244061931967735</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1749,7 +1749,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.04265908151865006</v>
+        <v>0.04244061931967735</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1775,7 +1775,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.03981514275074005</v>
+        <v>0.03961124271154404</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1801,7 +1801,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03981514275074005</v>
+        <v>0.03961124271154404</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1827,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03981514275074005</v>
+        <v>0.03961124271154404</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1853,7 +1853,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03981514275074005</v>
+        <v>0.03961124271154404</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1879,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.03697120398283005</v>
+        <v>0.03678186982870102</v>
       </c>
       <c r="C31" s="1">
         <v>26</v>
@@ -1905,7 +1905,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02559544891119003</v>
+        <v>0.02546437084674835</v>
       </c>
       <c r="C32" s="1">
         <v>18</v>
@@ -1931,7 +1931,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01421969383955002</v>
+        <v>0.01414687279611826</v>
       </c>
       <c r="C33" s="1">
         <v>10</v>
@@ -1957,7 +1957,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01137575507164002</v>
+        <v>0.01131749805063009</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1983,7 +1983,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01137575507164002</v>
+        <v>0.01131749805063009</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2009,7 +2009,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.005687877535820007</v>
+        <v>0.005658749025315046</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
add check uid function
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-3e4af7.o</t>
+    <t>lto-llvm-fe9c0b.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -243,7 +243,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-3e4af7.o</c:v>
+                  <c:v>lto-llvm-fe9c0b.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -261,10 +261,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>91.76518249511719</c:v>
+                  <c:v>91.77840423583984</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.234821319580078</c:v>
+                  <c:v>8.221597671508789</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -338,7 +338,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-3e4af7.o</c:v>
+                  <c:v>lto-llvm-fe9c0b.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -452,106 +452,106 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>94.00738525390625</c:v>
+                  <c:v>94.03791809082031</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.382333278656006</c:v>
+                  <c:v>2.370195150375366</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5715336799621582</c:v>
+                  <c:v>0.5686216354370117</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4725055396556854</c:v>
+                  <c:v>0.4700981080532074</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3282074630260468</c:v>
+                  <c:v>0.3265351951122284</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3225486874580383</c:v>
+                  <c:v>0.3209052979946137</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2631318271160126</c:v>
+                  <c:v>0.2617911696434021</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2489849627017975</c:v>
+                  <c:v>0.2477163672447205</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1556155979633331</c:v>
+                  <c:v>0.1548227220773697</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.141468733549118</c:v>
+                  <c:v>0.1407479345798492</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08771061152219772</c:v>
+                  <c:v>0.08726371824741364</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.07922248542308807</c:v>
+                  <c:v>0.07881884276866913</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07639311254024506</c:v>
+                  <c:v>0.07600388675928116</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07073436677455902</c:v>
+                  <c:v>0.07037396728992462</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.07073436677455902</c:v>
+                  <c:v>0.07037396728992462</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.06790498644113541</c:v>
+                  <c:v>0.06755901128053665</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.05658749118447304</c:v>
+                  <c:v>0.05629917234182358</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.05375811830163002</c:v>
+                  <c:v>0.05348421633243561</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.0509287416934967</c:v>
+                  <c:v>0.05066925659775734</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.0509287416934967</c:v>
+                  <c:v>0.05066925659775734</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04809936881065369</c:v>
+                  <c:v>0.04785429686307907</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.04526999220252037</c:v>
+                  <c:v>0.0450393408536911</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.04244061931967735</c:v>
+                  <c:v>0.04222438111901283</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.04244061931967735</c:v>
+                  <c:v>0.04222438111901283</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.03961124271154404</c:v>
+                  <c:v>0.03940942138433456</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03961124271154404</c:v>
+                  <c:v>0.03940942138433456</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03961124271154404</c:v>
+                  <c:v>0.03940942138433456</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03961124271154404</c:v>
+                  <c:v>0.03940942138433456</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.03678186982870102</c:v>
+                  <c:v>0.0365944616496563</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02546437084674835</c:v>
+                  <c:v>0.02533462829887867</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01414687279611826</c:v>
+                  <c:v>0.01407479308545589</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01131749805063009</c:v>
+                  <c:v>0.01125983521342278</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01131749805063009</c:v>
+                  <c:v>0.01125983521342278</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.005658749025315046</c:v>
+                  <c:v>0.005629917606711388</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -1018,16 +1018,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.76518249511719</v>
+        <v>91.77840423583984</v>
       </c>
       <c r="C3" s="1">
-        <v>11411</v>
+        <v>11431</v>
       </c>
       <c r="D3" s="1">
-        <v>66451</v>
+        <v>66813</v>
       </c>
       <c r="E3" s="1">
-        <v>66206</v>
+        <v>66568</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1036,7 +1036,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11256</v>
+        <v>11276</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1044,7 +1044,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.234821319580078</v>
+        <v>8.221597671508789</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1151,16 +1151,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>94.00738525390625</v>
+        <v>94.03791809082031</v>
       </c>
       <c r="C3" s="1">
-        <v>66451</v>
+        <v>66813</v>
       </c>
       <c r="D3" s="1">
-        <v>11411</v>
+        <v>11431</v>
       </c>
       <c r="E3" s="1">
-        <v>66206</v>
+        <v>66568</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1169,7 +1169,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11256</v>
+        <v>11276</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1177,7 +1177,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.382333278656006</v>
+        <v>2.370195150375366</v>
       </c>
       <c r="C4" s="1">
         <v>1684</v>
@@ -1203,7 +1203,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5715336799621582</v>
+        <v>0.5686216354370117</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.4725055396556854</v>
+        <v>0.4700981080532074</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1255,7 +1255,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.3282074630260468</v>
+        <v>0.3265351951122284</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1281,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3225486874580383</v>
+        <v>0.3209052979946137</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1307,7 +1307,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.2631318271160126</v>
+        <v>0.2617911696434021</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1333,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2489849627017975</v>
+        <v>0.2477163672447205</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1359,7 +1359,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1556155979633331</v>
+        <v>0.1548227220773697</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1385,7 +1385,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.141468733549118</v>
+        <v>0.1407479345798492</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1411,7 +1411,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08771061152219772</v>
+        <v>0.08726371824741364</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1437,7 +1437,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.07922248542308807</v>
+        <v>0.07881884276866913</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1463,7 +1463,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.07639311254024506</v>
+        <v>0.07600388675928116</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1489,7 +1489,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07073436677455902</v>
+        <v>0.07037396728992462</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1515,7 +1515,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.07073436677455902</v>
+        <v>0.07037396728992462</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1541,7 +1541,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.06790498644113541</v>
+        <v>0.06755901128053665</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1567,7 +1567,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.05658749118447304</v>
+        <v>0.05629917234182358</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.05375811830163002</v>
+        <v>0.05348421633243561</v>
       </c>
       <c r="C20" s="1">
         <v>38</v>
@@ -1619,7 +1619,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.0509287416934967</v>
+        <v>0.05066925659775734</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1645,7 +1645,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.0509287416934967</v>
+        <v>0.05066925659775734</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1671,7 +1671,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04809936881065369</v>
+        <v>0.04785429686307907</v>
       </c>
       <c r="C23" s="1">
         <v>34</v>
@@ -1697,7 +1697,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.04526999220252037</v>
+        <v>0.0450393408536911</v>
       </c>
       <c r="C24" s="1">
         <v>32</v>
@@ -1723,7 +1723,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.04244061931967735</v>
+        <v>0.04222438111901283</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1749,7 +1749,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.04244061931967735</v>
+        <v>0.04222438111901283</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1775,7 +1775,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.03961124271154404</v>
+        <v>0.03940942138433456</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1801,7 +1801,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03961124271154404</v>
+        <v>0.03940942138433456</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1827,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03961124271154404</v>
+        <v>0.03940942138433456</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1853,7 +1853,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03961124271154404</v>
+        <v>0.03940942138433456</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1879,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.03678186982870102</v>
+        <v>0.0365944616496563</v>
       </c>
       <c r="C31" s="1">
         <v>26</v>
@@ -1905,7 +1905,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02546437084674835</v>
+        <v>0.02533462829887867</v>
       </c>
       <c r="C32" s="1">
         <v>18</v>
@@ -1931,7 +1931,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01414687279611826</v>
+        <v>0.01407479308545589</v>
       </c>
       <c r="C33" s="1">
         <v>10</v>
@@ -1957,7 +1957,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01131749805063009</v>
+        <v>0.01125983521342278</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1983,7 +1983,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01131749805063009</v>
+        <v>0.01125983521342278</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2009,7 +2009,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.005658749025315046</v>
+        <v>0.005629917606711388</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
add ui updata flag
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-fe9c0b.o</t>
+    <t>lto-llvm-66c9e6.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -243,7 +243,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-fe9c0b.o</c:v>
+                  <c:v>lto-llvm-66c9e6.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -338,7 +338,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-fe9c0b.o</c:v>
+                  <c:v>lto-llvm-66c9e6.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -452,106 +452,106 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>94.03791809082031</c:v>
+                  <c:v>94.05565643310547</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.370195150375366</c:v>
+                  <c:v>2.363143920898438</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5686216354370117</c:v>
+                  <c:v>0.5669299960136414</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4700981080532074</c:v>
+                  <c:v>0.46869957447052</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3265351951122284</c:v>
+                  <c:v>0.3255637586116791</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3209052979946137</c:v>
+                  <c:v>0.3199506103992462</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2617911696434021</c:v>
+                  <c:v>0.2610123455524445</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2477163672447205</c:v>
+                  <c:v>0.2469794154167175</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1548227220773697</c:v>
+                  <c:v>0.1543621271848679</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1407479345798492</c:v>
+                  <c:v>0.1403292119503021</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08726371824741364</c:v>
+                  <c:v>0.08700411021709442</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.07881884276866913</c:v>
+                  <c:v>0.07858435809612274</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07600388675928116</c:v>
+                  <c:v>0.07577777653932571</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07037396728992462</c:v>
+                  <c:v>0.07016460597515106</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.07037396728992462</c:v>
+                  <c:v>0.07016460597515106</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.06755901128053665</c:v>
+                  <c:v>0.06735802441835403</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.05629917234182358</c:v>
+                  <c:v>0.05613168329000473</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.05348421633243561</c:v>
+                  <c:v>0.0533251017332077</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.05066925659775734</c:v>
+                  <c:v>0.05051851645112038</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.05066925659775734</c:v>
+                  <c:v>0.05051851645112038</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04785429686307907</c:v>
+                  <c:v>0.04771193116903305</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.0450393408536911</c:v>
+                  <c:v>0.04490534961223602</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.04222438111901283</c:v>
+                  <c:v>0.0420987643301487</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.04222438111901283</c:v>
+                  <c:v>0.0420987643301487</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.03940942138433456</c:v>
+                  <c:v>0.03929217904806137</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03940942138433456</c:v>
+                  <c:v>0.03929217904806137</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03940942138433456</c:v>
+                  <c:v>0.03929217904806137</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03940942138433456</c:v>
+                  <c:v>0.03929217904806137</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.0365944616496563</c:v>
+                  <c:v>0.03648559376597405</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02533462829887867</c:v>
+                  <c:v>0.02525925822556019</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01407479308545589</c:v>
+                  <c:v>0.01403292082250118</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01125983521342278</c:v>
+                  <c:v>0.01122633740305901</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01125983521342278</c:v>
+                  <c:v>0.01122633740305901</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.005629917606711388</c:v>
+                  <c:v>0.005613168701529503</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -1024,10 +1024,10 @@
         <v>11431</v>
       </c>
       <c r="D3" s="1">
-        <v>66813</v>
+        <v>67025</v>
       </c>
       <c r="E3" s="1">
-        <v>66568</v>
+        <v>66780</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1151,16 +1151,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>94.03791809082031</v>
+        <v>94.05565643310547</v>
       </c>
       <c r="C3" s="1">
-        <v>66813</v>
+        <v>67025</v>
       </c>
       <c r="D3" s="1">
         <v>11431</v>
       </c>
       <c r="E3" s="1">
-        <v>66568</v>
+        <v>66780</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1177,7 +1177,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.370195150375366</v>
+        <v>2.363143920898438</v>
       </c>
       <c r="C4" s="1">
         <v>1684</v>
@@ -1203,7 +1203,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5686216354370117</v>
+        <v>0.5669299960136414</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.4700981080532074</v>
+        <v>0.46869957447052</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1255,7 +1255,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.3265351951122284</v>
+        <v>0.3255637586116791</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1281,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3209052979946137</v>
+        <v>0.3199506103992462</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1307,7 +1307,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.2617911696434021</v>
+        <v>0.2610123455524445</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1333,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2477163672447205</v>
+        <v>0.2469794154167175</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1359,7 +1359,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1548227220773697</v>
+        <v>0.1543621271848679</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1385,7 +1385,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.1407479345798492</v>
+        <v>0.1403292119503021</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1411,7 +1411,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08726371824741364</v>
+        <v>0.08700411021709442</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1437,7 +1437,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.07881884276866913</v>
+        <v>0.07858435809612274</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1463,7 +1463,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.07600388675928116</v>
+        <v>0.07577777653932571</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1489,7 +1489,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07037396728992462</v>
+        <v>0.07016460597515106</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1515,7 +1515,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.07037396728992462</v>
+        <v>0.07016460597515106</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1541,7 +1541,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.06755901128053665</v>
+        <v>0.06735802441835403</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1567,7 +1567,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.05629917234182358</v>
+        <v>0.05613168329000473</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.05348421633243561</v>
+        <v>0.0533251017332077</v>
       </c>
       <c r="C20" s="1">
         <v>38</v>
@@ -1619,7 +1619,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.05066925659775734</v>
+        <v>0.05051851645112038</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1645,7 +1645,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.05066925659775734</v>
+        <v>0.05051851645112038</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1671,7 +1671,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04785429686307907</v>
+        <v>0.04771193116903305</v>
       </c>
       <c r="C23" s="1">
         <v>34</v>
@@ -1697,7 +1697,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.0450393408536911</v>
+        <v>0.04490534961223602</v>
       </c>
       <c r="C24" s="1">
         <v>32</v>
@@ -1723,7 +1723,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.04222438111901283</v>
+        <v>0.0420987643301487</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1749,7 +1749,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.04222438111901283</v>
+        <v>0.0420987643301487</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1775,7 +1775,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.03940942138433456</v>
+        <v>0.03929217904806137</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1801,7 +1801,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03940942138433456</v>
+        <v>0.03929217904806137</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1827,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03940942138433456</v>
+        <v>0.03929217904806137</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1853,7 +1853,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03940942138433456</v>
+        <v>0.03929217904806137</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1879,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.0365944616496563</v>
+        <v>0.03648559376597405</v>
       </c>
       <c r="C31" s="1">
         <v>26</v>
@@ -1905,7 +1905,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02533462829887867</v>
+        <v>0.02525925822556019</v>
       </c>
       <c r="C32" s="1">
         <v>18</v>
@@ -1931,7 +1931,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01407479308545589</v>
+        <v>0.01403292082250118</v>
       </c>
       <c r="C33" s="1">
         <v>10</v>
@@ -1957,7 +1957,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01125983521342278</v>
+        <v>0.01122633740305901</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1983,7 +1983,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01125983521342278</v>
+        <v>0.01122633740305901</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2009,7 +2009,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.005629917606711388</v>
+        <v>0.005613168701529503</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
fix cal temp flash data error
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-66c9e6.o</t>
+    <t>lto-llvm-b458e9.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -243,7 +243,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-66c9e6.o</c:v>
+                  <c:v>lto-llvm-b458e9.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -338,7 +338,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-66c9e6.o</c:v>
+                  <c:v>lto-llvm-b458e9.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>

</xml_diff>

<commit_message>
fix time show error,change key function
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-b458e9.o</t>
+    <t>lto-llvm-87d4b7.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -243,7 +243,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-b458e9.o</c:v>
+                  <c:v>lto-llvm-87d4b7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -261,10 +261,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>91.77840423583984</c:v>
+                  <c:v>91.77708435058594</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.221597671508789</c:v>
+                  <c:v>8.222918510437012</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -338,7 +338,7 @@
               <c:strCache>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-b458e9.o</c:v>
+                  <c:v>lto-llvm-87d4b7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -452,106 +452,106 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>94.05565643310547</c:v>
+                  <c:v>94.059326171875</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.363143920898438</c:v>
+                  <c:v>2.361685752868652</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5669299960136414</c:v>
+                  <c:v>0.5665801763534546</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.46869957447052</c:v>
+                  <c:v>0.4684103429317474</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3255637586116791</c:v>
+                  <c:v>0.325362890958786</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3199506103992462</c:v>
+                  <c:v>0.3197531700134277</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2610123455524445</c:v>
+                  <c:v>0.260851263999939</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2469794154167175</c:v>
+                  <c:v>0.2468270063400269</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1543621271848679</c:v>
+                  <c:v>0.1542668789625168</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1403292119503021</c:v>
+                  <c:v>0.1402426213026047</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08700411021709442</c:v>
+                  <c:v>0.08695042133331299</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.07858435809612274</c:v>
+                  <c:v>0.07853586971759796</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07577777653932571</c:v>
+                  <c:v>0.07573101669549942</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07016460597515106</c:v>
+                  <c:v>0.07012131065130234</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.07016460597515106</c:v>
+                  <c:v>0.07012131065130234</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.06735802441835403</c:v>
+                  <c:v>0.0673164576292038</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.05613168329000473</c:v>
+                  <c:v>0.05609704926609993</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.0533251017332077</c:v>
+                  <c:v>0.05329219624400139</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.05051851645112038</c:v>
+                  <c:v>0.05048734322190285</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.05051851645112038</c:v>
+                  <c:v>0.05048734322190285</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04771193116903305</c:v>
+                  <c:v>0.04768249019980431</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.04490534961223602</c:v>
+                  <c:v>0.04487763717770577</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.0420987643301487</c:v>
+                  <c:v>0.04207278415560722</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.0420987643301487</c:v>
+                  <c:v>0.04207278415560722</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.03929217904806137</c:v>
+                  <c:v>0.03926793485879898</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03929217904806137</c:v>
+                  <c:v>0.03926793485879898</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03929217904806137</c:v>
+                  <c:v>0.03926793485879898</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03929217904806137</c:v>
+                  <c:v>0.03926793485879898</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.03648559376597405</c:v>
+                  <c:v>0.03646308183670044</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02525925822556019</c:v>
+                  <c:v>0.02524367161095142</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01403292082250118</c:v>
+                  <c:v>0.01402426231652498</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01122633740305901</c:v>
+                  <c:v>0.01121940929442644</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01122633740305901</c:v>
+                  <c:v>0.01121940929442644</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.005613168701529503</c:v>
+                  <c:v>0.005609704647213221</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>0</c:v>
@@ -1018,16 +1018,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.77840423583984</v>
+        <v>91.77708435058594</v>
       </c>
       <c r="C3" s="1">
-        <v>11431</v>
+        <v>11429</v>
       </c>
       <c r="D3" s="1">
-        <v>67025</v>
+        <v>67069</v>
       </c>
       <c r="E3" s="1">
-        <v>66780</v>
+        <v>66824</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1036,7 +1036,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11276</v>
+        <v>11274</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1044,7 +1044,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.221597671508789</v>
+        <v>8.222918510437012</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1151,16 +1151,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>94.05565643310547</v>
+        <v>94.059326171875</v>
       </c>
       <c r="C3" s="1">
-        <v>67025</v>
+        <v>67069</v>
       </c>
       <c r="D3" s="1">
-        <v>11431</v>
+        <v>11429</v>
       </c>
       <c r="E3" s="1">
-        <v>66780</v>
+        <v>66824</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
@@ -1169,7 +1169,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11276</v>
+        <v>11274</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1177,7 +1177,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.363143920898438</v>
+        <v>2.361685752868652</v>
       </c>
       <c r="C4" s="1">
         <v>1684</v>
@@ -1203,7 +1203,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5669299960136414</v>
+        <v>0.5665801763534546</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.46869957447052</v>
+        <v>0.4684103429317474</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1255,7 +1255,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.3255637586116791</v>
+        <v>0.325362890958786</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1281,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3199506103992462</v>
+        <v>0.3197531700134277</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1307,7 +1307,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.2610123455524445</v>
+        <v>0.260851263999939</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1333,7 +1333,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2469794154167175</v>
+        <v>0.2468270063400269</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1359,7 +1359,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1543621271848679</v>
+        <v>0.1542668789625168</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1385,7 +1385,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.1403292119503021</v>
+        <v>0.1402426213026047</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1411,7 +1411,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08700411021709442</v>
+        <v>0.08695042133331299</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1437,7 +1437,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.07858435809612274</v>
+        <v>0.07853586971759796</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1463,7 +1463,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.07577777653932571</v>
+        <v>0.07573101669549942</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1489,7 +1489,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07016460597515106</v>
+        <v>0.07012131065130234</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1515,7 +1515,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.07016460597515106</v>
+        <v>0.07012131065130234</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1541,7 +1541,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.06735802441835403</v>
+        <v>0.0673164576292038</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1567,7 +1567,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.05613168329000473</v>
+        <v>0.05609704926609993</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.0533251017332077</v>
+        <v>0.05329219624400139</v>
       </c>
       <c r="C20" s="1">
         <v>38</v>
@@ -1619,7 +1619,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.05051851645112038</v>
+        <v>0.05048734322190285</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1645,7 +1645,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.05051851645112038</v>
+        <v>0.05048734322190285</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1671,7 +1671,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04771193116903305</v>
+        <v>0.04768249019980431</v>
       </c>
       <c r="C23" s="1">
         <v>34</v>
@@ -1697,7 +1697,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.04490534961223602</v>
+        <v>0.04487763717770577</v>
       </c>
       <c r="C24" s="1">
         <v>32</v>
@@ -1723,7 +1723,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.0420987643301487</v>
+        <v>0.04207278415560722</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1749,7 +1749,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.0420987643301487</v>
+        <v>0.04207278415560722</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1775,7 +1775,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.03929217904806137</v>
+        <v>0.03926793485879898</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1801,7 +1801,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03929217904806137</v>
+        <v>0.03926793485879898</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1827,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03929217904806137</v>
+        <v>0.03926793485879898</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1853,7 +1853,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03929217904806137</v>
+        <v>0.03926793485879898</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1879,7 +1879,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.03648559376597405</v>
+        <v>0.03646308183670044</v>
       </c>
       <c r="C31" s="1">
         <v>26</v>
@@ -1905,7 +1905,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02525925822556019</v>
+        <v>0.02524367161095142</v>
       </c>
       <c r="C32" s="1">
         <v>18</v>
@@ -1931,7 +1931,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01403292082250118</v>
+        <v>0.01402426231652498</v>
       </c>
       <c r="C33" s="1">
         <v>10</v>
@@ -1957,7 +1957,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01122633740305901</v>
+        <v>0.01121940929442644</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1983,7 +1983,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01122633740305901</v>
+        <v>0.01121940929442644</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2009,7 +2009,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.005613168701529503</v>
+        <v>0.005609704647213221</v>
       </c>
       <c r="C36" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
change max show temp to set temp when handle sleeping
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-87d4b7.o</t>
+    <t>lto-llvm-c4e36d.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>dcmpgt.o</t>
+  </si>
+  <si>
+    <t>dcmpge.o</t>
   </si>
   <si>
     <t>ffixi.o</t>
@@ -239,16 +242,16 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>ram_percent!$A$3:$A$37</c:f>
+              <c:f>ram_percent!$A$3:$A$38</c:f>
               <c:strCache>
-                <c:ptCount val="35"/>
+                <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-87d4b7.o</c:v>
+                  <c:v>lto-llvm-c4e36d.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="35">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -256,17 +259,17 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>ram_percent!$B$3:$B$37</c:f>
+              <c:f>ram_percent!$B$3:$B$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="35"/>
+                <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>91.77708435058594</c:v>
+                  <c:v>91.77972412109375</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.222918510437012</c:v>
-                </c:pt>
-                <c:pt idx="34">
+                  <c:v>8.220277786254883</c:v>
+                </c:pt>
+                <c:pt idx="35">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -334,11 +337,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>flash_percent!$A$3:$A$37</c:f>
+              <c:f>flash_percent!$A$3:$A$38</c:f>
               <c:strCache>
-                <c:ptCount val="35"/>
+                <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-87d4b7.o</c:v>
+                  <c:v>lto-llvm-c4e36d.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -377,69 +380,72 @@
                   <c:v>dcmpgt.o</c:v>
                 </c:pt>
                 <c:pt idx="13">
+                  <c:v>dcmpge.o</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>ffixi.o</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="15">
                   <c:v>dfixui.o</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="16">
                   <c:v>init.o</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="17">
                   <c:v>ffixui.o</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="18">
                   <c:v>f2d.o</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="19">
                   <c:v>memseta.o</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="20">
                   <c:v>llsshr.o</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="21">
                   <c:v>dflti.o</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="22">
                   <c:v>llushr.o</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="23">
                   <c:v>llshl.o</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="24">
                   <c:v>handlers.o</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="25">
                   <c:v>fcmplt.o</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="26">
                   <c:v>fcmple.o</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="27">
                   <c:v>fcmpgt.o</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="28">
                   <c:v>fcmpge.o</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="29">
                   <c:v>dfltui.o</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="30">
                   <c:v>fflti.o</c:v>
                 </c:pt>
-                <c:pt idx="30">
+                <c:pt idx="31">
                   <c:v>ffltui.o</c:v>
                 </c:pt>
-                <c:pt idx="31">
+                <c:pt idx="32">
                   <c:v>entry9a.o</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="33">
                   <c:v>entry2.o</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="34">
                   <c:v>entry5.o</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="35">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -447,113 +453,116 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>flash_percent!$B$3:$B$37</c:f>
+              <c:f>flash_percent!$B$3:$B$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="35"/>
+                <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>94.059326171875</c:v>
+                  <c:v>93.96263885498047</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.361685752868652</c:v>
+                  <c:v>2.415499210357666</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5665801763534546</c:v>
+                  <c:v>0.5614854097366333</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4684103429317474</c:v>
+                  <c:v>0.4641983509063721</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.325362890958786</c:v>
+                  <c:v>0.3224371671676636</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3197531700134277</c:v>
+                  <c:v>0.3168779313564301</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.260851263999939</c:v>
+                  <c:v>0.2585056722164154</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2468270063400269</c:v>
+                  <c:v>0.2446075230836868</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1542668789625168</c:v>
+                  <c:v>0.1528797000646591</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1402426213026047</c:v>
+                  <c:v>0.1389815360307694</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08695042133331299</c:v>
+                  <c:v>0.0861685574054718</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.07853586971759796</c:v>
+                  <c:v>0.07782966643571854</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07573101669549942</c:v>
+                  <c:v>0.07505003362894058</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07012131065130234</c:v>
+                  <c:v>0.07505003362894058</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.07012131065130234</c:v>
+                  <c:v>0.06949076801538467</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.0673164576292038</c:v>
+                  <c:v>0.06949076801538467</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.05609704926609993</c:v>
+                  <c:v>0.06671114265918732</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.05329219624400139</c:v>
+                  <c:v>0.0555926188826561</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.05048734322190285</c:v>
+                  <c:v>0.05281298607587814</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.05048734322190285</c:v>
+                  <c:v>0.05003335699439049</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04768249019980431</c:v>
+                  <c:v>0.05003335699439049</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.04487763717770577</c:v>
+                  <c:v>0.04725372418761253</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.04207278415560722</c:v>
+                  <c:v>0.04447409510612488</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.04207278415560722</c:v>
+                  <c:v>0.04169446229934692</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.03926793485879898</c:v>
+                  <c:v>0.04169446229934692</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03926793485879898</c:v>
+                  <c:v>0.03891483321785927</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03926793485879898</c:v>
+                  <c:v>0.03891483321785927</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03926793485879898</c:v>
+                  <c:v>0.03891483321785927</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.03646308183670044</c:v>
+                  <c:v>0.03891483321785927</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02524367161095142</c:v>
+                  <c:v>0.03613520041108131</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01402426231652498</c:v>
+                  <c:v>0.02501667849719524</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01121940929442644</c:v>
+                  <c:v>0.01389815472066402</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01121940929442644</c:v>
+                  <c:v>0.01111852377653122</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.005609704647213221</c:v>
+                  <c:v>0.01111852377653122</c:v>
                 </c:pt>
                 <c:pt idx="34">
+                  <c:v>0.00555926188826561</c:v>
+                </c:pt>
+                <c:pt idx="35">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -658,8 +667,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H37" totalsRowCount="1">
-  <autoFilter ref="A2:H36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H38" totalsRowCount="1">
+  <autoFilter ref="A2:H37"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="ram_percent" totalsRowFunction="sum"/>
@@ -675,8 +684,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H37" totalsRowCount="1">
-  <autoFilter ref="A2:H36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H38" totalsRowCount="1">
+  <autoFilter ref="A2:H37"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="flash_percent" totalsRowFunction="sum"/>
@@ -976,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -989,28 +998,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1018,25 +1027,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.77708435058594</v>
+        <v>91.77972412109375</v>
       </c>
       <c r="C3" s="1">
-        <v>11429</v>
+        <v>11433</v>
       </c>
       <c r="D3" s="1">
-        <v>67069</v>
+        <v>67608</v>
       </c>
       <c r="E3" s="1">
-        <v>66824</v>
+        <v>67362</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
       </c>
       <c r="G3" s="1">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H3" s="1">
-        <v>11274</v>
+        <v>11277</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1044,7 +1053,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.222918510437012</v>
+        <v>8.220277786254883</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1065,35 +1074,35 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37">
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
         <f>SUBTOTAL(109,[ram_percent])</f>
         <v>0</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="D37">
+      <c r="D38">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="E37">
+      <c r="E38">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F38">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G37">
+      <c r="G38">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H37">
+      <c r="H38">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>
@@ -1109,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1122,28 +1131,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
         <v>44</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1151,25 +1160,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>94.059326171875</v>
+        <v>93.96263885498047</v>
       </c>
       <c r="C3" s="1">
-        <v>67069</v>
+        <v>67608</v>
       </c>
       <c r="D3" s="1">
-        <v>11429</v>
+        <v>11433</v>
       </c>
       <c r="E3" s="1">
-        <v>66824</v>
+        <v>67362</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
       </c>
       <c r="G3" s="1">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H3" s="1">
-        <v>11274</v>
+        <v>11277</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1177,16 +1186,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.361685752868652</v>
+        <v>2.415499210357666</v>
       </c>
       <c r="C4" s="1">
-        <v>1684</v>
+        <v>1738</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <v>1684</v>
+        <v>1738</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
@@ -1203,7 +1212,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5665801763534546</v>
+        <v>0.5614854097366333</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1229,7 +1238,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.4684103429317474</v>
+        <v>0.4641983509063721</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1255,7 +1264,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.325362890958786</v>
+        <v>0.3224371671676636</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1281,7 +1290,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3197531700134277</v>
+        <v>0.3168779313564301</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1307,7 +1316,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.260851263999939</v>
+        <v>0.2585056722164154</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1333,7 +1342,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2468270063400269</v>
+        <v>0.2446075230836868</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1359,7 +1368,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1542668789625168</v>
+        <v>0.1528797000646591</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1385,7 +1394,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.1402426213026047</v>
+        <v>0.1389815360307694</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1411,7 +1420,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08695042133331299</v>
+        <v>0.0861685574054718</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1437,7 +1446,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.07853586971759796</v>
+        <v>0.07782966643571854</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1463,7 +1472,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.07573101669549942</v>
+        <v>0.07505003362894058</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1489,16 +1498,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07012131065130234</v>
+        <v>0.07505003362894058</v>
       </c>
       <c r="C16" s="1">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1515,7 +1524,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.07012131065130234</v>
+        <v>0.06949076801538467</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1541,16 +1550,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.0673164576292038</v>
+        <v>0.06949076801538467</v>
       </c>
       <c r="C18" s="1">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -1567,16 +1576,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.05609704926609993</v>
+        <v>0.06671114265918732</v>
       </c>
       <c r="C19" s="1">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
       </c>
       <c r="E19" s="1">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -1593,16 +1602,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.05329219624400139</v>
+        <v>0.0555926188826561</v>
       </c>
       <c r="C20" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -1619,16 +1628,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.05048734322190285</v>
+        <v>0.05281298607587814</v>
       </c>
       <c r="C21" s="1">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D21" s="1">
         <v>0</v>
       </c>
       <c r="E21" s="1">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -1645,7 +1654,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.05048734322190285</v>
+        <v>0.05003335699439049</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1671,16 +1680,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04768249019980431</v>
+        <v>0.05003335699439049</v>
       </c>
       <c r="C23" s="1">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D23" s="1">
         <v>0</v>
       </c>
       <c r="E23" s="1">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -1697,16 +1706,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.04487763717770577</v>
+        <v>0.04725372418761253</v>
       </c>
       <c r="C24" s="1">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D24" s="1">
         <v>0</v>
       </c>
       <c r="E24" s="1">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -1723,16 +1732,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.04207278415560722</v>
+        <v>0.04447409510612488</v>
       </c>
       <c r="C25" s="1">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -1749,7 +1758,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.04207278415560722</v>
+        <v>0.04169446229934692</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1775,16 +1784,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.03926793485879898</v>
+        <v>0.04169446229934692</v>
       </c>
       <c r="C27" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D27" s="1">
         <v>0</v>
       </c>
       <c r="E27" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
@@ -1801,7 +1810,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03926793485879898</v>
+        <v>0.03891483321785927</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1827,7 +1836,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03926793485879898</v>
+        <v>0.03891483321785927</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1853,7 +1862,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03926793485879898</v>
+        <v>0.03891483321785927</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1879,16 +1888,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.03646308183670044</v>
+        <v>0.03891483321785927</v>
       </c>
       <c r="C31" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D31" s="1">
         <v>0</v>
       </c>
       <c r="E31" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
@@ -1905,16 +1914,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02524367161095142</v>
+        <v>0.03613520041108131</v>
       </c>
       <c r="C32" s="1">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D32" s="1">
         <v>0</v>
       </c>
       <c r="E32" s="1">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -1931,16 +1940,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01402426231652498</v>
+        <v>0.02501667849719524</v>
       </c>
       <c r="C33" s="1">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D33" s="1">
         <v>0</v>
       </c>
       <c r="E33" s="1">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -1957,16 +1966,16 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01121940929442644</v>
+        <v>0.01389815472066402</v>
       </c>
       <c r="C34" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D34" s="1">
         <v>0</v>
       </c>
       <c r="E34" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -1983,7 +1992,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01121940929442644</v>
+        <v>0.01111852377653122</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2009,56 +2018,82 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.005609704647213221</v>
+        <v>0.01111852377653122</v>
       </c>
       <c r="C36" s="1">
+        <v>8</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1">
+        <v>8</v>
+      </c>
+      <c r="F36" s="1">
+        <v>0</v>
+      </c>
+      <c r="G36" s="1">
+        <v>0</v>
+      </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="2">
+        <v>0.00555926188826561</v>
+      </c>
+      <c r="C37" s="1">
         <v>4</v>
       </c>
-      <c r="D36" s="1">
-        <v>0</v>
-      </c>
-      <c r="E36" s="1">
+      <c r="D37" s="1">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1">
         <v>4</v>
       </c>
-      <c r="F36" s="1">
-        <v>0</v>
-      </c>
-      <c r="G36" s="1">
-        <v>0</v>
-      </c>
-      <c r="H36" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37">
+      <c r="F37" s="1">
+        <v>0</v>
+      </c>
+      <c r="G37" s="1">
+        <v>0</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
         <f>SUBTOTAL(109,[flash_percent])</f>
         <v>0</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="D37">
+      <c r="D38">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="E37">
+      <c r="E38">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F38">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G37">
+      <c r="G38">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H37">
+      <c r="H38">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
add curve page bace on last commit
</commit_message>
<xml_diff>
--- a/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/G1/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-444d48.o</t>
+    <t>lto-llvm-b72985.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -246,7 +246,7 @@
               <c:strCache>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-444d48.o</c:v>
+                  <c:v>lto-llvm-b72985.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -264,10 +264,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>91.78104400634766</c:v>
+                  <c:v>91.78367614746094</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.218957901000977</c:v>
+                  <c:v>8.216320037841797</c:v>
                 </c:pt>
                 <c:pt idx="35">
                   <c:v>0</c:v>
@@ -341,7 +341,7 @@
               <c:strCache>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-444d48.o</c:v>
+                  <c:v>lto-llvm-b72985.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -458,109 +458,109 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="36"/>
                 <c:pt idx="0">
-                  <c:v>93.99319458007813</c:v>
+                  <c:v>94.00885772705078</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.403274536132813</c:v>
+                  <c:v>2.39700984954834</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5586437582969666</c:v>
+                  <c:v>0.557187557220459</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4618490636348724</c:v>
+                  <c:v>0.4606451690196991</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3208053410053253</c:v>
+                  <c:v>0.319969117641449</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3152742087841034</c:v>
+                  <c:v>0.3144524097442627</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.257197380065918</c:v>
+                  <c:v>0.2565269470214844</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2433695644140244</c:v>
+                  <c:v>0.2427351772785187</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1521059721708298</c:v>
+                  <c:v>0.1517094969749451</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.1382781565189362</c:v>
+                  <c:v>0.1379177123308182</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.08573246002197266</c:v>
+                  <c:v>0.08550898730754852</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.07743576914072037</c:v>
+                  <c:v>0.0772339254617691</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07467020303010941</c:v>
+                  <c:v>0.07447557151317596</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.07467020303010941</c:v>
+                  <c:v>0.07447557151317596</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.06913907825946808</c:v>
+                  <c:v>0.06895885616540909</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.06913907825946808</c:v>
+                  <c:v>0.06895885616540909</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.06637351959943771</c:v>
+                  <c:v>0.06620050221681595</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.05531126260757446</c:v>
+                  <c:v>0.05516708642244339</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.0525457002222538</c:v>
+                  <c:v>0.05240873247385025</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.04978013783693314</c:v>
+                  <c:v>0.04965037852525711</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.04978013783693314</c:v>
+                  <c:v>0.04965037852525711</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.04701457545161247</c:v>
+                  <c:v>0.04689202457666397</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.04424901306629181</c:v>
+                  <c:v>0.04413367062807083</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.04148344695568085</c:v>
+                  <c:v>0.04137531667947769</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.04148344695568085</c:v>
+                  <c:v>0.04137531667947769</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.03871788457036018</c:v>
+                  <c:v>0.03861696273088455</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.03871788457036018</c:v>
+                  <c:v>0.03861696273088455</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.03871788457036018</c:v>
+                  <c:v>0.03861696273088455</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.03871788457036018</c:v>
+                  <c:v>0.03861696273088455</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.03595232218503952</c:v>
+                  <c:v>0.03585860505700111</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.02489006891846657</c:v>
+                  <c:v>0.02482518926262856</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01382781565189362</c:v>
+                  <c:v>0.01379177160561085</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01106225326657295</c:v>
+                  <c:v>0.01103341765701771</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.01106225326657295</c:v>
+                  <c:v>0.01103341765701771</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.005531126633286476</c:v>
+                  <c:v>0.005516708828508854</c:v>
                 </c:pt>
                 <c:pt idx="35">
                   <c:v>0</c:v>
@@ -1027,25 +1027,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.78104400634766</v>
+        <v>91.78367614746094</v>
       </c>
       <c r="C3" s="1">
-        <v>11435</v>
+        <v>11439</v>
       </c>
       <c r="D3" s="1">
-        <v>67974</v>
+        <v>68163</v>
       </c>
       <c r="E3" s="1">
-        <v>67728</v>
+        <v>67916</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
       </c>
       <c r="G3" s="1">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H3" s="1">
-        <v>11279</v>
+        <v>11282</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1053,7 +1053,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.218957901000977</v>
+        <v>8.216320037841797</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1160,25 +1160,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>93.99319458007813</v>
+        <v>94.00885772705078</v>
       </c>
       <c r="C3" s="1">
-        <v>67974</v>
+        <v>68163</v>
       </c>
       <c r="D3" s="1">
-        <v>11435</v>
+        <v>11439</v>
       </c>
       <c r="E3" s="1">
-        <v>67728</v>
+        <v>67916</v>
       </c>
       <c r="F3" s="1">
         <v>90</v>
       </c>
       <c r="G3" s="1">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H3" s="1">
-        <v>11279</v>
+        <v>11282</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1186,7 +1186,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.403274536132813</v>
+        <v>2.39700984954834</v>
       </c>
       <c r="C4" s="1">
         <v>1738</v>
@@ -1212,7 +1212,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.5586437582969666</v>
+        <v>0.557187557220459</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1238,7 +1238,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.4618490636348724</v>
+        <v>0.4606451690196991</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1264,7 +1264,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.3208053410053253</v>
+        <v>0.319969117641449</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1290,7 +1290,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.3152742087841034</v>
+        <v>0.3144524097442627</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1316,7 +1316,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.257197380065918</v>
+        <v>0.2565269470214844</v>
       </c>
       <c r="C9" s="1">
         <v>186</v>
@@ -1342,7 +1342,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.2433695644140244</v>
+        <v>0.2427351772785187</v>
       </c>
       <c r="C10" s="1">
         <v>176</v>
@@ -1368,7 +1368,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.1521059721708298</v>
+        <v>0.1517094969749451</v>
       </c>
       <c r="C11" s="1">
         <v>110</v>
@@ -1394,7 +1394,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.1382781565189362</v>
+        <v>0.1379177123308182</v>
       </c>
       <c r="C12" s="1">
         <v>100</v>
@@ -1420,7 +1420,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.08573246002197266</v>
+        <v>0.08550898730754852</v>
       </c>
       <c r="C13" s="1">
         <v>62</v>
@@ -1446,7 +1446,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.07743576914072037</v>
+        <v>0.0772339254617691</v>
       </c>
       <c r="C14" s="1">
         <v>56</v>
@@ -1472,7 +1472,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.07467020303010941</v>
+        <v>0.07447557151317596</v>
       </c>
       <c r="C15" s="1">
         <v>54</v>
@@ -1498,7 +1498,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.07467020303010941</v>
+        <v>0.07447557151317596</v>
       </c>
       <c r="C16" s="1">
         <v>54</v>
@@ -1524,7 +1524,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.06913907825946808</v>
+        <v>0.06895885616540909</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1550,7 +1550,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.06913907825946808</v>
+        <v>0.06895885616540909</v>
       </c>
       <c r="C18" s="1">
         <v>50</v>
@@ -1576,7 +1576,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.06637351959943771</v>
+        <v>0.06620050221681595</v>
       </c>
       <c r="C19" s="1">
         <v>48</v>
@@ -1602,7 +1602,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.05531126260757446</v>
+        <v>0.05516708642244339</v>
       </c>
       <c r="C20" s="1">
         <v>40</v>
@@ -1628,7 +1628,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.0525457002222538</v>
+        <v>0.05240873247385025</v>
       </c>
       <c r="C21" s="1">
         <v>38</v>
@@ -1654,7 +1654,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.04978013783693314</v>
+        <v>0.04965037852525711</v>
       </c>
       <c r="C22" s="1">
         <v>36</v>
@@ -1680,7 +1680,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.04978013783693314</v>
+        <v>0.04965037852525711</v>
       </c>
       <c r="C23" s="1">
         <v>36</v>
@@ -1706,7 +1706,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.04701457545161247</v>
+        <v>0.04689202457666397</v>
       </c>
       <c r="C24" s="1">
         <v>34</v>
@@ -1732,7 +1732,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.04424901306629181</v>
+        <v>0.04413367062807083</v>
       </c>
       <c r="C25" s="1">
         <v>32</v>
@@ -1758,7 +1758,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.04148344695568085</v>
+        <v>0.04137531667947769</v>
       </c>
       <c r="C26" s="1">
         <v>30</v>
@@ -1784,7 +1784,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.04148344695568085</v>
+        <v>0.04137531667947769</v>
       </c>
       <c r="C27" s="1">
         <v>30</v>
@@ -1810,7 +1810,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.03871788457036018</v>
+        <v>0.03861696273088455</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1836,7 +1836,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.03871788457036018</v>
+        <v>0.03861696273088455</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1862,7 +1862,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.03871788457036018</v>
+        <v>0.03861696273088455</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1888,7 +1888,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.03871788457036018</v>
+        <v>0.03861696273088455</v>
       </c>
       <c r="C31" s="1">
         <v>28</v>
@@ -1914,7 +1914,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.03595232218503952</v>
+        <v>0.03585860505700111</v>
       </c>
       <c r="C32" s="1">
         <v>26</v>
@@ -1940,7 +1940,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.02489006891846657</v>
+        <v>0.02482518926262856</v>
       </c>
       <c r="C33" s="1">
         <v>18</v>
@@ -1966,7 +1966,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01382781565189362</v>
+        <v>0.01379177160561085</v>
       </c>
       <c r="C34" s="1">
         <v>10</v>
@@ -1992,7 +1992,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01106225326657295</v>
+        <v>0.01103341765701771</v>
       </c>
       <c r="C35" s="1">
         <v>8</v>
@@ -2018,7 +2018,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.01106225326657295</v>
+        <v>0.01103341765701771</v>
       </c>
       <c r="C36" s="1">
         <v>8</v>
@@ -2044,7 +2044,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="2">
-        <v>0.005531126633286476</v>
+        <v>0.005516708828508854</v>
       </c>
       <c r="C37" s="1">
         <v>4</v>

</xml_diff>